<commit_message>
used: Finish-LP and OM
</commit_message>
<xml_diff>
--- a/Open-LPs.xlsx
+++ b/Open-LPs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B75"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,606 +443,554 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LP-042605</t>
+          <t>LP-049701</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Encerrado!</t>
+          <t>Compromisso pendente!</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LP-045880</t>
+          <t>LP-049802</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Encerrado!</t>
+          <t>Compromisso pendente!</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LP-046158</t>
+          <t>LP-049808</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Encerrado!</t>
+          <t>Compromisso pendente!</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LP-048214</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>LP-049869</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Compromisso pendente!</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LP-048388</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>LP-049986</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LP-048523</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>LP-050022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LP-048524</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>LP-050074</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LP-048853</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>LP-050101</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LP-048852</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>LP-050107</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LP-048995</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>LP-050221</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LP-049083</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>LP-050265</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LP-049171</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>LP-050288</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LP-049174</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>LP-050289</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LP-049176</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>LP-050291</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LP-049233</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>LP-050295</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LP-049294</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>LP-050306</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LP-049537</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>LP-050307</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LP-049557</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
+          <t>LP-050329</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LP-049592</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>LP-050330</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LP-049701</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>LP-050340</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LP-049713</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>LP-050345</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LP-049719</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+          <t>LP-050346</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LP-049802</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>LP-050362</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LP-049808</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
+          <t>LP-050481</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LP-049869</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>LP-050492</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LP-049920</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>LP-050558</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Compromisso pendente!</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LP-049925</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>LP-050559</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Compromisso pendente!</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LP-049926</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>LP-050575</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LP-049927</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>LP-050843</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Compromisso pendente!</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LP-049949</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>LP-043689</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LP-049951</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>LP-045882</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LP-049981</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t>LP-047197</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LP-049986</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
+          <t>LP-048173</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LP-050022</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
+          <t>LP-048269</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LP-050074</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t>LP-048512</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LP-050101</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
+          <t>LP-049045</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LP-050107</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
+          <t>LP-049296</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LP-050221</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
+          <t>LP-049317</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LP-050265</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
+          <t>LP-049374</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LP-050288</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
+          <t>LP-049390</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LP-050289</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
+          <t>LP-049503</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LP-050291</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
+          <t>LP-049649</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LP-050295</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
+          <t>LP-049665</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LP-050306</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
+          <t>LP-049756</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LP-050307</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t>LP-049863</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LP-050329</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>LP-050330</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>LP-050340</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>LP-050345</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>LP-050346</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>LP-050362</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>LP-050481</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>LP-050492</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>LP-050558</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>LP-050559</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>LP-050575</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>LP-050843</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>LP-043689</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>LP-045882</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>LP-047197</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>LP-048173</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>LP-048269</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>LP-048512</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>LP-049045</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>LP-049296</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>LP-049317</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>LP-049374</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>LP-049390</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>LP-049503</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>LP-049649</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>LP-049665</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>LP-049756</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>LP-049863</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
           <t>LP-050157</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Encerrado!</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
used: finish bot lp and om
</commit_message>
<xml_diff>
--- a/Open-LPs.xlsx
+++ b/Open-LPs.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F98D75-2AD1-4127-88FE-C0B36325D05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A31D3C-1616-44CA-A654-BAB3A1B75121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$50</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="51">
   <si>
     <t>LP</t>
   </si>
@@ -88,6 +85,9 @@
     <t>LP-050498</t>
   </si>
   <si>
+    <t>LP-050151</t>
+  </si>
+  <si>
     <t>LP-050598</t>
   </si>
   <si>
@@ -163,9 +163,6 @@
     <t>LP-051251</t>
   </si>
   <si>
-    <t>LP-051259</t>
-  </si>
-  <si>
     <t>LP-051350</t>
   </si>
   <si>
@@ -176,9 +173,6 @@
   </si>
   <si>
     <t>LP-051537</t>
-  </si>
-  <si>
-    <t>LP-050151</t>
   </si>
 </sst>
 </file>
@@ -541,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -702,157 +696,188 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>51</v>
+        <v>39</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>41</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>44</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>45</v>
+      </c>
+      <c r="B26" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>46</v>
+      </c>
+      <c r="B27" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>47</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>48</v>
+      </c>
+      <c r="B29" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>49</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>50</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>